<commit_message>
Builder M2: export SCORM package (streaming zip) + Workday info
- src/zip.js: own streaming zip writer; video STORED, text DEFLATE. Writes the
  header first and patches CRC/sizes afterwards (no data descriptors), so Java's
  ZipInputStream can read it. Blocks packages over 4 GB.
- src/package.js: course.js + imsmanifest.xml + player files, mirroring build()
  in build_scorm.py; disk sink (showSaveFilePicker, Chrome/Edge) and in-memory
  fallback for other browsers (< 500 MB)
- Step 5 UI: export button, MB progress, Workday fields with copy buttons
- Tests: package equivalence with build_scorm.py (node), export via disk and
  memory paths in Chromium, optional LARGE=1 1.5 GB export; Player 26/26 on
  the Builder-made package
- Template 'Hướng dẫn' sheet links to the Builder; docs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DkjQ94JxW9pMDUqdRVGGx
</commit_message>
<xml_diff>
--- a/demo-course/ATLD-DEMO.xlsx
+++ b/demo-course/ATLD-DEMO.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -561,88 +561,88 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Đóng gói</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ô nền vàng nhạt là ô cần điền. Không đổi tên sheet, không đổi tiêu đề cột.</t>
+          <t>Điền xong, mở https://ctd-academy.github.io/scorm/ bằng Chrome hoặc Edge, chọn file Excel + thư mục video, bấm Xuất gói SCORM</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sheet 'Thông tin khóa': thông tin chung và luật bài kiểm tra của khóa.</t>
+          <t>Ô nền vàng nhạt là ô cần điền. Không đổi tên sheet, không đổi tiêu đề cột.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sheet 'Video': mỗi dòng là 1 bài (1 video), theo đúng thứ tự học. Tên file phải trùng tên file video trong thư mục khóa.</t>
+          <t>Sheet 'Thông tin khóa': thông tin chung và luật bài kiểm tra của khóa.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sheet 'Câu hỏi': gồm cả câu hỏi pop-up (giữa video) và câu hỏi bài kiểm tra cuối khóa.</t>
+          <t>Sheet 'Video': mỗi dòng là 1 bài (1 video), theo đúng thứ tự học. Tên file phải trùng tên file video trong thư mục khóa.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Sheet 'Câu hỏi': gồm cả câu hỏi pop-up (giữa video) và câu hỏi bài kiểm tra cuối khóa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Dòng 2 ở mỗi sheet (chữ nghiêng) là VÍ DỤ. Xóa hoặc ghi đè khi nhập khóa thật.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Luật chơi cố định</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Học tuần tự: bài sau chỉ mở khi xem xong bài trước.</t>
-        </is>
-      </c>
+      <c r="B12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Video chỉ tua lại phần đã xem, không tua tới. Tốc độ tối đa 2x. Rời trang/chuyển tab thì video tự dừng.</t>
+          <t>Học tuần tự: bài sau chỉ mở khi xem xong bài trước.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Pop-up không tính điểm. Trả lời sai thì phải xem lại đoạn video trước câu hỏi (từ pop-up trước đó, hoặc từ đầu video).</t>
+          <t>Video chỉ tua lại phần đã xem, không tua tới. Tốc độ tối đa 2x. Rời trang/chuyển tab thì video tự dừng.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Bài kiểm tra chỉ mở khi đã xem hết video. Khóa không có câu hỏi CUỐI KHÓA sẽ hoàn thành khi xem hết video.</t>
+          <t>Pop-up không tính điểm. Trả lời sai thì phải xem lại đoạn video trước câu hỏi (từ pop-up trước đó, hoặc từ đầu video).</t>
         </is>
       </c>
     </row>
@@ -688,129 +688,129 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>Bài kiểm tra chỉ mở khi đã xem hết video. Khóa không có câu hỏi CUỐI KHÓA sẽ hoàn thành khi xem hết video.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>Hết lượt làm bài: bài kiểm tra bị khóa, học viên thấy nội dung liên hệ L&amp;OD. L&amp;OD đăng ký lại cho học viên trên Workday.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Quy ước nhập câu hỏi</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Loại</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>POPUP = câu hỏi giữa video · CUOI KHOA = câu hỏi bài kiểm tra cuối khóa</t>
-        </is>
-      </c>
+      <c r="B19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Video số</t>
+          <t>Loại</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Chỉ điền cho POPUP: số thứ tự bài (cột STT ở sheet Video)</t>
+          <t>POPUP = câu hỏi giữa video · CUOI KHOA = câu hỏi bài kiểm tra cuối khóa</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Mốc thời gian</t>
+          <t>Video số</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Chỉ điền cho POPUP: phút:giây trong video, ví dụ 01:30. Nên đặt cách nhau ít nhất 1 phút</t>
+          <t>Chỉ điền cho POPUP: số thứ tự bài (cột STT ở sheet Video)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Phương án</t>
+          <t>Mốc thời gian</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tối thiểu A, B. C và D có thể bỏ trống</t>
+          <t>Chỉ điền cho POPUP: phút:giây trong video, ví dụ 01:30. Nên đặt cách nhau ít nhất 1 phút</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Đáp án đúng</t>
+          <t>Phương án</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Một chữ cái: A, B, C hoặc D</t>
+          <t>Tối thiểu A, B. C và D có thể bỏ trống</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Giải thích</t>
+          <t>Đáp án đúng</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Không bắt buộc. Hiện sau khi trả lời pop-up đúng, và khi xem lại bài kiểm tra (nếu bật hiện đáp án)</t>
+          <t>Một chữ cái: A, B, C hoặc D</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
+          <t>Giải thích</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Không bắt buộc. Hiện sau khi trả lời pop-up đúng, và khi xem lại bài kiểm tra (nếu bật hiện đáp án)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>Xáo phương án</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Thứ tự phương án được xáo mỗi lần thi. Dùng được 'Tất cả đều đúng', tránh viết 'Cả A và B đều đúng'</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Cài đặt bài kiểm tra (sheet 'Thông tin khóa')</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Gợi ý</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Điểm đạt 80% · 3 lượt · rút 15–20 câu từ ngân hàng 20–30 câu để mỗi lượt có đề khác nhau</t>
-        </is>
-      </c>
+      <c r="B28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -820,33 +820,33 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
+          <t>Điểm đạt 80% · 3 lượt · rút 15–20 câu từ ngân hàng 20–30 câu để mỗi lượt có đề khác nhau</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Gợi ý</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
           <t>Thời gian làm bài: khoảng 1–1,5 phút cho mỗi câu. Hiện đáp án: nên chọn 'Không' để người rớt không học thuộc đáp án cho lượt sau</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="3" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Cách viết câu hỏi pop-up</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Mục đích là giữ học viên tập trung, không đánh đố. Hỏi đúng điều vừa nói trong 1–2 phút trước mốc</t>
-        </is>
-      </c>
+      <c r="B32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Đặt mốc ngay sau khi ý chính kết thúc. Khoảng 1 câu cho mỗi 3–5 phút video, cách nhau ít nhất 1 phút</t>
+          <t>Mục đích là giữ học viên tập trung, không đánh đố. Hỏi đúng điều vừa nói trong 1–2 phút trước mốc</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Không đặt trong 30 giây đầu hoặc ở cuối video. 2–3 phương án ngắn là đủ. Nên có Giải thích</t>
+          <t>Đặt mốc ngay sau khi ý chính kết thúc. Khoảng 1 câu cho mỗi 3–5 phút video, cách nhau ít nhất 1 phút</t>
         </is>
       </c>
     </row>
@@ -880,17 +880,29 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
+          <t>Không đặt trong 30 giây đầu hoặc ở cuối video. 2–3 phương án ngắn là đủ. Nên có Giải thích</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
           <t>Không dùng lại câu hỏi cuối khóa làm pop-up</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Ô cần điền</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>